<commit_message>
feat: add branch name to environment config and enhance company registration data model
</commit_message>
<xml_diff>
--- a/test_cases/eDOT_QA_Automation_Test_Cases.xlsx
+++ b/test_cases/eDOT_QA_Automation_Test_Cases.xlsx
@@ -184,7 +184,7 @@
       </c>
       <c r="B3" t="inlineStr" s="2">
         <is>
-          <t>Register Company Step 1 keeps Next disabled until required data is valid</t>
+          <t>Register Company Step 1 keeps Next disabled until required dependent data is valid</t>
         </is>
       </c>
       <c r="C3" t="inlineStr" s="2">
@@ -194,17 +194,17 @@
       </c>
       <c r="D3" t="inlineStr" s="2">
         <is>
-          <t>1. Leave Step 1 fields blank; 2. Confirm Next is disabled; 3. Fill Company Name only; 4. Confirm Next remains disabled; 5. Fill all required Step 1 fields including dependent location cascade; 6. Confirm Next becomes enabled.</t>
+          <t>1. Leave Step 1 fields blank; 2. Confirm Next is disabled; 3. Select Country only; 4. Confirm downstream mandatory cascade fields remain disabled until their parent value is selected; 5. Fill all required Step 1 fields in order: Country, Province, City/District, District/Commune, Sub District/Village; 6. Confirm Postal Code is auto-populated from the selected village/sub-district; 7. Confirm Next becomes enabled only after all required values are complete.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr" s="2">
         <is>
-          <t>Company Name=PT Nusantara Ritel Mandiri QA ${RUN_ID}; Email=qa.company+${RUN_ID}@example.test; Phone=+6281234567890; Industry Type=Retail; Company Type=Retailer; Language=English; Street Address=Jl. Sudirman No. 10; Country=Indonesia; Province=DKI Jakarta; City=Jakarta Selatan; District=Kebayoran Baru; Zone=Senayan; Postal Code=12190</t>
+          <t>Company Name=PT Nusantara Ritel Mandiri QA ${RUN_ID}; Email=qa${RUN_ID}@qa.test; Phone=81234567890; Industry Type=Retail; Company Type=Retailer; Language=English; Street Address=Jl. Sudirman No. 10; Country=Indonesia; Province=DKI Jakarta; City/District=Jakarta Selatan; District/Commune=Kebayoran Baru; Sub District/Village=Senayan; Postal Code=12190</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="2">
         <is>
-          <t>Next button remains disabled while any required Step 1 field or cascade value is missing, and becomes enabled only after all listed values are valid. No error text is expected before submit because assignment specifies disabled state.</t>
+          <t>Before parent cascade values are selected, mandatory dependent fields are disabled and Next remains disabled. After the cascade is completed in order, Postal Code may remain read-only but must show the expected auto-filled value, and Next must become enabled.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr" s="2">
@@ -236,12 +236,12 @@
       </c>
       <c r="D4" t="inlineStr" s="2">
         <is>
-          <t>1. Open Companies; 2. Click + Add Company; 3. Complete Step 1 with validated AI company data or deterministic fallback data; 4. Complete Steps 2 and 3 using only required product fields; 5. Submit registration; 6. Open Companies to Manage and search exact Company Name.</t>
+          <t>1. Open Companies; 2. Click + Add Company; 3. Complete Step 1 with validated AI company data or deterministic fallback data; 4. Continue through optional Step 2; 5. Complete Step 3 Branch Name and terms checkbox; 6. Submit registration; 7. Open Companies to Manage and search exact Company Name.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr" s="2">
         <is>
-          <t>Company Name=PT Nusantara Ritel Mandiri QA ${RUN_ID}; Email=qa.company+${RUN_ID}@example.test; Phone=+6281234567890; Industry Type=Retail; Company Type=Retailer; Language=English; Street Address=Jl. Sudirman No. 10; Country=Indonesia; Province=DKI Jakarta; City=Jakarta Selatan; District=Kebayoran Baru; Zone=Senayan; Postal Code=12190; Step 2 and Step 3=&lt;minimum required product fields discovered during implementation&gt;</t>
+          <t>Company Name=PT Nusantara Ritel Mandiri QA ${RUN_ID}; Email=qa${RUN_ID}@qa.test; Phone=81234567890; Industry Type=Retail; Company Type=Retailer; Language=English; Street Address=Jl. Sudirman No. 10; Country=Indonesia; Province=DKI Jakarta; City=Jakarta Selatan; District=Kebayoran Baru; Zone/Sub District=Senayan; Postal Code=12190; Branch Name=Main; Terms and Conditions=checked</t>
         </is>
       </c>
       <c r="F4" t="inlineStr" s="2">

</xml_diff>

<commit_message>
Refactor and clean up eDOT QA Automation project
- Deleted outdated implementation plan and codex automation plan files.
- Updated README to reflect current project status and verification notes.
- Improved allure reporting helpers by removing console step prints.
- Enhanced RegisterCompanyWizardPage with more robust success notification checks.
- Cleaned up debug timing script and removed it from the repository.
- Updated package.json for better allure report cleanup commands.
- Modified manual test cases Excel file metadata for clarity.
- Improved test quality gate checks to include additional ignored directories.
</commit_message>
<xml_diff>
--- a/test_cases/eDOT_QA_Automation_Test_Cases.xlsx
+++ b/test_cases/eDOT_QA_Automation_Test_Cases.xlsx
@@ -472,12 +472,12 @@
     <row r="3" ht="28" customHeight="1">
       <c r="A3" t="inlineStr" s="2">
         <is>
-          <t>Execution framework</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="B3" t="inlineStr" s="2">
         <is>
-          <t>edot_codex_qa_automation_plan.md</t>
+          <t>eDOT QA Automation Take-Home V4</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: update test case IDs and add additional test case tags for consistency in manual test cases
</commit_message>
<xml_diff>
--- a/test_cases/eDOT_QA_Automation_Test_Cases.xlsx
+++ b/test_cases/eDOT_QA_Automation_Test_Cases.xlsx
@@ -194,22 +194,22 @@
       </c>
       <c r="D3" t="inlineStr" s="2">
         <is>
-          <t>1. Leave Step 1 fields blank; 2. Confirm Next is disabled; 3. Select Country only; 4. Confirm downstream mandatory cascade fields remain disabled until their parent value is selected; 5. Fill all required Step 1 fields in order: Country, Province, City/District, District/Commune, Sub District/Village; 6. Confirm Postal Code is auto-populated from the selected village/sub-district; 7. Confirm Next becomes enabled only after all required values are complete.</t>
+          <t>1. Leave Step 1 fields blank; 2. Confirm Next is disabled; 3. Fill required fields in visible form order: Company Name, Email, Phone, Industry Type, Company Type, Language, Street Address, Country; 4. Complete dependent location cascade in order: Country, Province, City/District, District/Commune, Sub District/Village; 5. Confirm Postal Code is auto-populated from the selected village/sub-district; 6. Confirm Next becomes enabled only after all required values are complete.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr" s="2">
         <is>
-          <t>Company Name=PT Nusantara Ritel Mandiri QA ${RUN_ID}; Email=qa${RUN_ID}@qa.test; Phone=81234567890; Industry Type=Retail; Company Type=Retailer; Language=English; Street Address=Jl. Sudirman No. 10; Country=Indonesia; Province=DKI Jakarta; City/District=Jakarta Selatan; District/Commune=Kebayoran Baru; Sub District/Village=Senayan; Postal Code=12190</t>
+          <t>Canonical sample / runtime generated in Allure: Company Name=PT Ritel QA ${RUN_ID}; Email=qa.company.${RUN_ID}@example.test; Phone=81234567890; Industry Type=Retail; Company Type=Retailer; Language=English; Street Address=Jalan Sudirman No 10; Country=Indonesia; Province=DKI Jakarta; City/District=Jakarta Selatan; District/Commune=Kebayoran Baru; Sub District/Village=Senayan; Postal Code=12190</t>
         </is>
       </c>
       <c r="F3" t="inlineStr" s="2">
         <is>
-          <t>Before parent cascade values are selected, mandatory dependent fields are disabled and Next remains disabled. After the cascade is completed in order, Postal Code may remain read-only but must show the expected auto-filled value, and Next must become enabled.</t>
+          <t>Before required values are complete, mandatory dependent fields remain unavailable as designed and Next remains disabled. After the cascade is completed in order, Postal Code may remain read-only but must show the expected auto-filled value, and Next must become enabled.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr" s="2">
         <is>
-          <t>Negative</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="H3" t="inlineStr" s="2">
@@ -241,7 +241,7 @@
       </c>
       <c r="E4" t="inlineStr" s="2">
         <is>
-          <t>Company Name=PT Nusantara Ritel Mandiri QA ${RUN_ID}; Email=qa${RUN_ID}@qa.test; Phone=81234567890; Industry Type=Retail; Company Type=Retailer; Language=English; Street Address=Jl. Sudirman No. 10; Country=Indonesia; Province=DKI Jakarta; City=Jakarta Selatan; District=Kebayoran Baru; Zone/Sub District=Senayan; Postal Code=12190; Branch Name=Main; Terms and Conditions=checked</t>
+          <t>Canonical sample / runtime generated in Allure: Company Name=PT Ritel QA ${RUN_ID}; Email=qa.company.${RUN_ID}@example.test; Phone=81234567890; Industry Type=Retail; Company Type=Retailer; Language=English; Street Address=Jalan Sudirman No 10; Country=Indonesia; Province=DKI Jakarta; City=Jakarta Selatan; District=Kebayoran Baru; Zone/Sub District=Senayan; Postal Code=12190; Branch Name=Main; Terms and Conditions=checked</t>
         </is>
       </c>
       <c r="F4" t="inlineStr" s="2">
@@ -273,22 +273,22 @@
       </c>
       <c r="C5" t="inlineStr" s="2">
         <is>
-          <t>Company from WEB-TC-003 exists and its exact input data is available from the test run.</t>
+          <t>Company from WEB-TC-003 exists and the exact submitted input payload is attached to the same Allure run.</t>
         </is>
       </c>
       <c r="D5" t="inlineStr" s="2">
         <is>
-          <t>1. Open Companies; 2. Open Manage; 3. Search exact Company Name; 4. Open company detail; 5. Compare every required detail field with the submitted value.</t>
+          <t>1. Open Companies; 2. Open Manage; 3. Search exact Company Name from WEB-TC-003; 4. Open company detail; 5. Compare every required detail field with the submitted value from WEB-TC-003.</t>
         </is>
       </c>
       <c r="E5" t="inlineStr" s="2">
         <is>
-          <t>Company Name=PT Nusantara Ritel Mandiri QA ${RUN_ID}; Email=qa.company+${RUN_ID}@example.test; Phone=+6281234567890; Industry Type=Retail; Company Type=Retailer; Street Address=Jl. Sudirman No. 10; Postal Code=12190</t>
+          <t>Same submitted values from WEB-TC-003: Company Name=PT Ritel QA ${RUN_ID}; Email=qa.company.${RUN_ID}@example.test; Phone=81234567890; Industry Type=Retail; Company Type=Retailer; Street Address=Jalan Sudirman No 10; Postal Code=12190</t>
         </is>
       </c>
       <c r="F5" t="inlineStr" s="2">
         <is>
-          <t>Detail view values equal submitted values for name, industry type, company type, address, postal code, email, and phone.</t>
+          <t>Detail view values equal submitted values from WEB-TC-003 for name, industry type, company type, address, postal code, email, and phone.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr" s="2">
@@ -320,17 +320,17 @@
       </c>
       <c r="D6" t="inlineStr" s="2">
         <is>
-          <t>1. Open Companies; 2. Open Manage; 3. Search exact Company Name; 4. Delete the company; 5. Confirm deletion; 6. Search exact Company Name again.</t>
+          <t>1. Open Companies; 2. Open Manage; 3. Search exact Company Name and captured Company ID from WEB-TC-003; 4. Delete the company; 5. Confirm deletion; 6. Search exact Company Name and Company ID again.</t>
         </is>
       </c>
       <c r="E6" t="inlineStr" s="2">
         <is>
-          <t>Company Name=PT Nusantara Ritel Mandiri QA ${RUN_ID}</t>
+          <t>Company Name=PT Ritel QA ${RUN_ID}; Company ID=&lt;captured non-secret runtime value&gt;</t>
         </is>
       </c>
       <c r="F6" t="inlineStr" s="2">
         <is>
-          <t>Company is removed from Manage results and cannot be opened from search. Shared environment has no leftover company for current RUN_ID.</t>
+          <t>Company name and captured Company ID are removed from Manage results and cannot be opened from search. Shared environment has no leftover company for current RUN_ID.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr" s="2">

</xml_diff>

<commit_message>
feat: add mobile customer case validation test and update test cases for accuracy
</commit_message>
<xml_diff>
--- a/test_cases/eDOT_QA_Automation_Test_Cases.xlsx
+++ b/test_cases/eDOT_QA_Automation_Test_Cases.xlsx
@@ -352,27 +352,27 @@
       </c>
       <c r="B7" t="inlineStr" s="2">
         <is>
-          <t>Login to eWork SFA using newly created company credentials</t>
+          <t>Login to eWork SFA with company user credentials</t>
         </is>
       </c>
       <c r="C7" t="inlineStr" s="2">
         <is>
-          <t>eWork SFA is installed; emulator or device is visible in adb devices; mobile credentials are supplied through environment variables; prefer company created by web run.</t>
+          <t>eWork SFA is installed; emulator or physical device is visible in adb devices; Maestro CLI is available; mobile credentials are supplied through environment variables; prefer Company User created under the web-created company, otherwise use the assignment fallback only if documented.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr" s="2">
         <is>
-          <t>1. Launch eWork SFA; 2. Run reusable login flow; 3. Enter EWORK_COMPANY_ID; 4. Enter EWORK_USERNAME; 5. Enter EWORK_PASSWORD; 6. Submit login.</t>
+          <t>1. Launch eWork SFA; 2. Run reusable login sub-flow; 3. Enter EWORK_COMPANY_CODE from web-created company or fallback env; 4. Enter EWORK_USERNAME / Company User username; 5. Enter EWORK_PASSWORD from secure env; 6. Tap Sign In; 7. Wait for dashboard text.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr" s="2">
         <is>
-          <t>EWORK_COMPANY_ID=&lt;company created by web run&gt;; EWORK_USERNAME=&lt;secure environment value&gt;; EWORK_PASSWORD=&lt;secure environment value&gt;</t>
+          <t>EWORK_COMPANY_CODE=&lt;web-created company ID/code or fallback env&gt;; EWORK_USERNAME=&lt;company user username from web handoff or secure env&gt;; EWORK_PASSWORD=&lt;secure environment value&gt;; EWORK_STORAGE_STATE=&lt;non-secret local session marker&gt;</t>
         </is>
       </c>
       <c r="F7" t="inlineStr" s="2">
         <is>
-          <t>Mobile dashboard is displayed after login.</t>
+          <t>Mobile dashboard is displayed after login and the reusable app session can be consumed by non-login mobile tests.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr" s="2">
@@ -394,27 +394,27 @@
       </c>
       <c r="B8" t="inlineStr" s="2">
         <is>
-          <t>Create a customer in eWork SFA with AI-generated Indonesian customer data</t>
+          <t>Create a customer in eWork SFA and verify the saved card values</t>
         </is>
       </c>
       <c r="C8" t="inlineStr" s="2">
         <is>
-          <t>User is logged in to eWork SFA; customer data has passed schema validation or deterministic fallback generation.</t>
+          <t>User is logged in to eWork SFA using reusable app session; customer data has passed AI schema validation or deterministic fallback generation; device location permission is available; no customer exists for current RUN_ID.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr" s="2">
         <is>
-          <t>1. Open customer module; 2. Add new customer; 3. Fill customer name, contact, and address; 4. Save; 5. Search or open created customer; 6. Compare displayed values with input data.</t>
+          <t>1. Open New Customer menu; 2. Tap New Customer Registration; 3. Basic tab: enter Outlet Name, Contact, and Contact Person; 4. Select Channel and Customer Type; 5. Continue to Locations; 6. Select Address Type; 7. Tap Use my current location; 8. Assert Address field is auto-filled and capture that displayed address; 9. Select Province, City, District, Sub District, and Postal Code in order; 10. Continue to Documents; 11. Enter 16 digit KTP number; 12. Tap Upload File and capture any camera image; 13. Submit document; 14. Draw signature line; 15. Tap Register/Save and confirm; 16. Assert success message; 17. Return to New Customer List; 18. Validate the customer card directly if visible, otherwise fast-scroll to the bottom, then search upward at most four slow swipes.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr" s="2">
         <is>
-          <t>Customer Name=Budi Santoso QA ${RUN_ID}; Contact=+6281299900111; Address=Jl. Melati Raya No. 8, Kebayoran Baru, Jakarta Selatan 12190</t>
+          <t>Customer Name=Budi Santoso QA ${RUN_ID}; Contact=+6281299900111; Contact Person=Raka QA PIC ${RUN_ID}; Channel=Modern Trade (MT); Customer Type=Semi Grosir; Address Type=Delivery Address; Current Location Address=&lt;captured from app address field&gt;; Province=DKI JAKARTA; City=JAKARTA BARAT; District=KEBON JERUK; Sub District=KEBON JERUK; Postal Code=11530; KTP=&lt;16 digit runtime value&gt;; Attachment=camera capture; Signature=drawn</t>
         </is>
       </c>
       <c r="F8" t="inlineStr" s="2">
         <is>
-          <t>Created customer appears in the customer list/detail, and displayed name, contact, and address equal the submitted values.</t>
+          <t>Created customer appears on New Customer List card. Card name equals submitted Outlet Name, card address equals the address captured from the app after Use my current location, and card customer type equals submitted Customer Type. If the card is not found after bottom validation plus four upward searches, the test fails.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr" s="2">

</xml_diff>